<commit_message>
093025 - added a 2025 handicaps file for use next year
</commit_message>
<xml_diff>
--- a/public/results/2024 Handicaps.xlsx
+++ b/public/results/2024 Handicaps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F6CFBE0-2AB0-864B-A284-481C141E9CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68DE52E-184B-4C47-9054-BFD9D4558CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8540" yWindow="2580" windowWidth="24720" windowHeight="16440" xr2:uid="{64927184-4E58-1140-B742-9AE1581050D8}"/>
+    <workbookView xWindow="345" yWindow="15" windowWidth="19830" windowHeight="10785" xr2:uid="{64927184-4E58-1140-B742-9AE1581050D8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
-    <t>end 2024 handicaps</t>
-  </si>
-  <si>
     <t>Arndt</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t>Young</t>
+  </si>
+  <si>
+    <t>End 2024 handicaps</t>
   </si>
 </sst>
 </file>
@@ -514,164 +514,164 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C330AA6-8EBE-5748-92A7-85B1B0621E10}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="C2" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="C3" s="2">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="C4" s="2">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C6" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="C7" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C8" s="2">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C9" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C10" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C11" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="2">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C13" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C14" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2">
         <v>13</v>

</xml_diff>